<commit_message>
Creacion de 2 packs iniciales
</commit_message>
<xml_diff>
--- a/src/data/xlsx/data.xlsx
+++ b/src/data/xlsx/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cristobal\Desarrollo\mindsolut\src\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23D5A808-8B6E-4231-9AAE-F4EA3DCDA35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9DF5E7-03C4-40D9-93CC-A6E905976CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{499745C3-64F6-4343-B2DD-22AAF1801A63}"/>
+    <workbookView xWindow="32190" yWindow="3270" windowWidth="21600" windowHeight="11235" activeTab="4" xr2:uid="{499745C3-64F6-4343-B2DD-22AAF1801A63}"/>
   </bookViews>
   <sheets>
     <sheet name="Topics" sheetId="4" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2979,13 +2979,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5021,7 +5020,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F630CCB9-A219-454F-BCD7-F728987A49D8}" name="TablaDinámica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" colHeaderCaption="Is Premium">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F630CCB9-A219-454F-BCD7-F728987A49D8}" name="TablaDinámica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" colHeaderCaption="Is Premium">
   <location ref="A4:D11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -5873,10 +5872,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>950</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="4"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -5904,11 +5903,10 @@
       <c r="A6" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6">
         <v>25</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3">
+      <c r="D6">
         <v>25</v>
       </c>
     </row>
@@ -5916,11 +5914,10 @@
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7">
         <v>24</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3">
+      <c r="D7">
         <v>24</v>
       </c>
     </row>
@@ -5928,11 +5925,10 @@
       <c r="A8" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8">
         <v>35</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3">
+      <c r="D8">
         <v>35</v>
       </c>
     </row>
@@ -5940,11 +5936,10 @@
       <c r="A9" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9">
         <v>35</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3">
+      <c r="D9">
         <v>35</v>
       </c>
     </row>
@@ -5952,13 +5947,13 @@
       <c r="A10" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10">
         <v>10</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10">
         <v>10</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10">
         <v>20</v>
       </c>
     </row>
@@ -5966,13 +5961,13 @@
       <c r="A11" s="2" t="s">
         <v>948</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11">
         <v>129</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11">
         <v>10</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11">
         <v>139</v>
       </c>
     </row>
@@ -11747,7 +11742,9 @@
   <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="27.6640625" customWidth="1"/>
     <col min="2" max="2" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
     <col min="4" max="4" width="11.88671875" customWidth="1"/>
     <col min="10" max="10" width="12.21875" customWidth="1"/>
     <col min="12" max="12" width="18.5546875" customWidth="1"/>

</xml_diff>